<commit_message>
Se agrega PCB MEC-V1.0 RevD - Enviado a fabricar a JLCPCB
</commit_message>
<xml_diff>
--- a/hardware/dev/Project Outputs for MEC/assembly files/MEC-V1.0-BoM JLCPCB.xlsx
+++ b/hardware/dev/Project Outputs for MEC/assembly files/MEC-V1.0-BoM JLCPCB.xlsx
@@ -16,612 +16,594 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="196">
+  <si>
+    <t>Designator</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>JLCPCB Part #</t>
+  </si>
   <si>
     <t>Description</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Designator</t>
-  </si>
-  <si>
-    <t>JLCPCB Part #</t>
+    <t>C1, C2, C3, C6, C7, C8, C9, C10, C17, C18, C19, C20, C21, C22, C23, C24</t>
+  </si>
+  <si>
+    <t>C107137</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 100 V 0.022 uF X7R 0805 10%</t>
   </si>
   <si>
-    <t>C1, C2, C3, C6, C7, C8, C9, C10, C17, C18, C19, C20, C21, C22, C23, C24</t>
-  </si>
-  <si>
-    <t>C107137</t>
+    <t>C4, C28, C41, C42, C43, C45, C46, C48, C49, C50, C51, C54, C57, C64, C65, C66, C67, C72, C73, C74, C75, C76</t>
+  </si>
+  <si>
+    <t>C105882</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 0.1uF X7R 0402 10%</t>
   </si>
   <si>
-    <t>C4, C28, C41, C42, C43, C45, C46, C48, C49, C50, C51, C54, C57, C64, C65, C66, C67, C72, C73, C74, C75, C76</t>
-  </si>
-  <si>
-    <t>C105882</t>
-  </si>
-  <si>
-    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 100 V 0.033 uF X7R 1206 10%</t>
-  </si>
-  <si>
     <t>C5</t>
   </si>
   <si>
-    <t>C113901</t>
+    <t>C327114</t>
+  </si>
+  <si>
+    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 100 V 0.033 uF X7R 0805 10%</t>
+  </si>
+  <si>
+    <t>C11, C12, C13, C14, C25, C34, C35, C36, C37</t>
+  </si>
+  <si>
+    <t>C107005</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 33 pF C0G 0402 1%</t>
   </si>
   <si>
-    <t>C11, C12, C13, C14, C25, C34, C35, C36, C37</t>
-  </si>
-  <si>
-    <t>C107005</t>
+    <t>C15, C52</t>
+  </si>
+  <si>
+    <t>C7500380</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50V 1uF X5R 0402 10% HI CV</t>
   </si>
   <si>
-    <t>C15, C52</t>
-  </si>
-  <si>
-    <t>C7500380</t>
+    <t>C16, C33, C38, C39, C40</t>
+  </si>
+  <si>
+    <t>C281751</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 100pF X7R 0402 10%</t>
   </si>
   <si>
-    <t>C16, C33, C38, C39, C40</t>
-  </si>
-  <si>
-    <t>C281751</t>
+    <t>C26</t>
+  </si>
+  <si>
+    <t>C107026</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 0.022uF X7R 0402 10%</t>
   </si>
   <si>
-    <t>C26</t>
-  </si>
-  <si>
-    <t>C107026</t>
+    <t>C27, C29, C30</t>
+  </si>
+  <si>
+    <t>C60133</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 0.01uF X7R 0402 10%</t>
   </si>
   <si>
-    <t>C27, C29, C30</t>
-  </si>
-  <si>
-    <t>C60133</t>
+    <t>C31</t>
+  </si>
+  <si>
+    <t>C513552</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 0.470uF X7R 0402 10%</t>
   </si>
   <si>
-    <t>C31</t>
-  </si>
-  <si>
-    <t>C513552</t>
+    <t>C32, C71</t>
+  </si>
+  <si>
+    <t>C326586</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 10V 4.7uF X5R 0402 10% HI CV</t>
   </si>
   <si>
-    <t>C32, C71</t>
-  </si>
-  <si>
-    <t>C326586</t>
+    <t>C53</t>
+  </si>
+  <si>
+    <t>C106207</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 470pF X7R 0402 10%</t>
   </si>
   <si>
-    <t>C53</t>
-  </si>
-  <si>
-    <t>C106207</t>
-  </si>
-  <si>
-    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 5.6pF C0G 0402 Tol 0.1pF</t>
-  </si>
-  <si>
-    <t>C55, C56, C70, C79</t>
-  </si>
-  <si>
-    <t>C505468</t>
+    <t>C55, C56, C68, C69, C70, C79</t>
+  </si>
+  <si>
+    <t>C326662</t>
+  </si>
+  <si>
+    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 12 pF C0G 0402 1%</t>
+  </si>
+  <si>
+    <t>C58, C63</t>
+  </si>
+  <si>
+    <t>C89827</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 16V 10uF X5R 0805 10%</t>
   </si>
   <si>
-    <t>C58, C63</t>
-  </si>
-  <si>
-    <t>C77075</t>
-  </si>
-  <si>
-    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 3kV 1000pF X7R 1812 10%</t>
-  </si>
-  <si>
     <t>C60</t>
   </si>
   <si>
-    <t>C577351</t>
+    <t>C23631</t>
+  </si>
+  <si>
+    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 2kV 1000pF X7R 1206 10%</t>
+  </si>
+  <si>
+    <t>C61, C62</t>
+  </si>
+  <si>
+    <t>C2897302</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50V 4.7uF X5R 0805 10%</t>
   </si>
   <si>
-    <t>C61, C62</t>
-  </si>
-  <si>
-    <t>C2897302</t>
-  </si>
-  <si>
-    <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 50 V 12 pF C0G 0402 1%</t>
-  </si>
-  <si>
-    <t>C68, C69</t>
-  </si>
-  <si>
-    <t>C326662</t>
+    <t>C77, C78</t>
+  </si>
+  <si>
+    <t>C723363</t>
   </si>
   <si>
     <t>Multilayer Ceramic Capacitors MLCC - SMD/SMT 25V 2.2uF X5R 0402 10% HI CV</t>
   </si>
   <si>
-    <t>C77, C78</t>
-  </si>
-  <si>
-    <t>C723363</t>
+    <t>D1, D2, D3, D4, D5, D6, D7, D8, D13, D14, D15, D16, D17, D18, D19, D20, D22, D36</t>
+  </si>
+  <si>
+    <t>C125094</t>
   </si>
   <si>
     <t>Standard Single Color LEDs 0603 Green</t>
   </si>
   <si>
-    <t>D1, D2, D3, D4, D5, D6, D7, D8, D13, D14, D15, D16, D17, D18, D19, D20, D22, D36</t>
-  </si>
-  <si>
-    <t>C125094</t>
+    <t>D9, D10, D11, D34</t>
+  </si>
+  <si>
+    <t>C94869</t>
   </si>
   <si>
     <t>Standard Single Color LEDs 0603 Red</t>
   </si>
   <si>
-    <t>D9, D10, D11, D34</t>
-  </si>
-  <si>
-    <t>C94869</t>
+    <t>D12, D28</t>
+  </si>
+  <si>
+    <t>C181204</t>
   </si>
   <si>
     <t>Schottky Diodes &amp; Rectifiers 350mA 40V SOD123</t>
   </si>
   <si>
-    <t>D12, D28</t>
-  </si>
-  <si>
-    <t>C181204</t>
+    <t>D21</t>
+  </si>
+  <si>
+    <t>C5122012</t>
   </si>
   <si>
     <t>ESD Protection Diodes / TVS Diodes SOT-23 7V400W Low Capacitance</t>
   </si>
   <si>
-    <t>D21</t>
-  </si>
-  <si>
-    <t>C5122012</t>
+    <t>D23, D35</t>
+  </si>
+  <si>
+    <t>C125095</t>
   </si>
   <si>
     <t>Standard Single Color LEDs 0603 Yellow</t>
   </si>
   <si>
-    <t>D23, D35</t>
-  </si>
-  <si>
-    <t>C125095</t>
+    <t>D24</t>
+  </si>
+  <si>
+    <t>C558419</t>
   </si>
   <si>
     <t>ESD Protection Diodes / TVS Diodes Low Cap ESD Protect</t>
   </si>
   <si>
-    <t>D24</t>
-  </si>
-  <si>
-    <t>C558419</t>
+    <t>D25, D26</t>
+  </si>
+  <si>
+    <t>C14996</t>
   </si>
   <si>
     <t>Schottky Diodes &amp; Rectifiers 2A 100V SMA</t>
   </si>
   <si>
-    <t>D25, D26</t>
-  </si>
-  <si>
-    <t>C14996</t>
+    <t>D27</t>
+  </si>
+  <si>
+    <t>C173517</t>
   </si>
   <si>
     <t>ESD Protection Diodes / TVS Diodes 400W 26V 5% Bi-Directional</t>
   </si>
   <si>
-    <t>D27</t>
-  </si>
-  <si>
-    <t>C173517</t>
+    <t>D29, D30, D31, D32, D33, D37</t>
+  </si>
+  <si>
+    <t>C19829399</t>
   </si>
   <si>
     <t>ESD Protection Diodes / TVS Diodes UNIDIRECTIONAL 3.3V ESD PR</t>
   </si>
   <si>
-    <t>D29, D30, D31, D32, D33, D37</t>
-  </si>
-  <si>
-    <t>C19829399</t>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>C136354</t>
   </si>
   <si>
     <t>Surface Mount Fuses 1206 high-current met-foil. 10A</t>
   </si>
   <si>
-    <t>F1</t>
-  </si>
-  <si>
-    <t>C136354</t>
+    <t>J9, J10, J11, J12, J15, J16, J17, J18, J24</t>
+  </si>
+  <si>
+    <t>C8475</t>
   </si>
   <si>
     <t>Pluggable Terminal Blocks 2 Pos 5.08mm pitch Through Hole Header</t>
   </si>
   <si>
-    <t>J9, J10, J11, J12, J15, J16, J17, J18, J24</t>
-  </si>
-  <si>
-    <t>C8475</t>
+    <t>J20</t>
+  </si>
+  <si>
+    <t>C8483</t>
   </si>
   <si>
     <t>Pluggable Terminal Blocks 3 Pos 5.08mm pitch Through Hole Header</t>
   </si>
   <si>
-    <t>J20</t>
-  </si>
-  <si>
-    <t>C8483</t>
+    <t>J22</t>
+  </si>
+  <si>
+    <t>C34677</t>
   </si>
   <si>
     <t>Modular Ethernet Connector Jack (Female) 1x1 Shielded Through Hole With LEDs With Magnetics</t>
   </si>
   <si>
-    <t>J22</t>
-  </si>
-  <si>
-    <t>C34677</t>
+    <t>J26</t>
+  </si>
+  <si>
+    <t>C7465995</t>
   </si>
   <si>
     <t>Male straight header, 2 row, 14 positions, 1.27mm pitch, SMD</t>
   </si>
   <si>
-    <t>J26</t>
-  </si>
-  <si>
-    <t>C7465995</t>
+    <t>J27</t>
+  </si>
+  <si>
+    <t>C192300</t>
   </si>
   <si>
     <t>Male straight header, 2 row, 8 positions, 2.54mm pitch, SMD</t>
   </si>
   <si>
-    <t>J27</t>
-  </si>
-  <si>
-    <t>C192300</t>
+    <t>L1</t>
+  </si>
+  <si>
+    <t>C83471</t>
   </si>
   <si>
     <t>Power Inductors - SMD 100uH 0.42A 1.6Ohms</t>
   </si>
   <si>
-    <t>L1</t>
-  </si>
-  <si>
-    <t>C83471</t>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>C76886</t>
   </si>
   <si>
     <t>Ferrite Beads 600 OHM 25% Alternate Sizing Guide Below</t>
   </si>
   <si>
-    <t>L2</t>
-  </si>
-  <si>
-    <t>C76886</t>
+    <t>L4</t>
+  </si>
+  <si>
+    <t>C878356</t>
   </si>
   <si>
     <t>Common Mode Chokes / Filters WE-SL2 SMD Sectional 2x10uH 1600mA</t>
   </si>
   <si>
-    <t>L4</t>
-  </si>
-  <si>
-    <t>C878356</t>
-  </si>
-  <si>
-    <t>Thick Film Resistors - SMD 2.2 kOhms 125 mW 0805 1%</t>
-  </si>
-  <si>
     <t>R1, R2, R5, R6, R7, R8, R9, R11</t>
   </si>
   <si>
     <t>C114561</t>
   </si>
   <si>
-    <t>Thick Film Resistors - SMD 1 kOhms 250 mW 1206 1%</t>
+    <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0805, 2.2kOhms, 1%, 1/8W</t>
   </si>
   <si>
     <t>R3</t>
   </si>
   <si>
-    <t>C131398</t>
+    <t>C95781</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0805, 1kOhms, 1%, 1/8W</t>
+  </si>
+  <si>
+    <t>R4</t>
+  </si>
+  <si>
+    <t>C107229</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 51kOhms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R4</t>
-  </si>
-  <si>
-    <t>C107229</t>
+    <t>R10</t>
+  </si>
+  <si>
+    <t>C114761</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 15kOhms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R10</t>
-  </si>
-  <si>
-    <t>C114761</t>
-  </si>
-  <si>
-    <t>Thick Film Resistors - SMD 1.5 MOhms 250 mW 1206 1%</t>
-  </si>
-  <si>
     <t>R12</t>
   </si>
   <si>
-    <t>C137367</t>
-  </si>
-  <si>
-    <t>Thick Film Resistors - SMD 120 kOhms 250 mW 1206 1%</t>
+    <t>C107700</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0805, 1MOhms, 1%, 1/8W</t>
   </si>
   <si>
     <t>R13</t>
   </si>
   <si>
-    <t>C163387</t>
+    <t>C137489</t>
+  </si>
+  <si>
+    <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0805, 82 kOhms, 1%, 1/8W</t>
+  </si>
+  <si>
+    <t>R14, R15, R16, R17, R21, R25, R26, R27, R28</t>
+  </si>
+  <si>
+    <t>C112291</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 220Ohms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R14, R15, R16, R17, R21, R25, R26, R27, R28</t>
-  </si>
-  <si>
-    <t>C112291</t>
+    <t>R18, R19, R20, R29, R30, R31, R35, R36, R37, R38, R39</t>
+  </si>
+  <si>
+    <t>C137948</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 680Ohms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R18, R19, R20, R29, R30, R31, R35, R36, R37, R38, R39</t>
-  </si>
-  <si>
-    <t>C137948</t>
+    <t>R22</t>
+  </si>
+  <si>
+    <t>C105576</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0603, 2kOhms, 1%, 1/10W</t>
   </si>
   <si>
-    <t>R22</t>
-  </si>
-  <si>
-    <t>C105576</t>
+    <t>R23</t>
+  </si>
+  <si>
+    <t>C98220</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0603, 10kOhms, 1%, 1/10W</t>
   </si>
   <si>
-    <t>R23</t>
-  </si>
-  <si>
-    <t>C98220</t>
+    <t>R24</t>
+  </si>
+  <si>
+    <t>C108078</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0603, 3.3kOhms, 1%, 1/10W</t>
   </si>
   <si>
-    <t>R24</t>
-  </si>
-  <si>
-    <t>C108078</t>
+    <t>R32, R33, R34, R40, R43, R44, R53, R54, R55, R56, R65, R72, R79</t>
+  </si>
+  <si>
+    <t>C60490</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 10kOhms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R32, R33, R34, R40, R43, R44, R53, R54, R55, R56, R65, R72, R79</t>
-  </si>
-  <si>
-    <t>C60490</t>
-  </si>
-  <si>
-    <t>Thick Film Resistors - SMD 0.5W 10ohms 1% High Power AEC-Q200</t>
-  </si>
-  <si>
     <t>R41, R45</t>
   </si>
   <si>
     <t>C844598</t>
   </si>
   <si>
+    <t>Thick Film Resistors - SMD High Power Chip Resistor 0805, 10Ohms, 1%, 1/2W</t>
+  </si>
+  <si>
+    <t>R42</t>
+  </si>
+  <si>
+    <t>C114758</t>
+  </si>
+  <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 120Ohms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R42</t>
-  </si>
-  <si>
-    <t>C114758</t>
+    <t>R46, R47</t>
+  </si>
+  <si>
+    <t>C106235</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 1kOhms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R46, R47</t>
-  </si>
-  <si>
-    <t>C106235</t>
+    <t>R49, R50, R51, R52</t>
+  </si>
+  <si>
+    <t>C87044</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 49.9Ohms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R49, R50, R51, R52</t>
-  </si>
-  <si>
-    <t>C87044</t>
+    <t>R57</t>
+  </si>
+  <si>
+    <t>C114759</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 1.5kOhms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R57</t>
-  </si>
-  <si>
-    <t>C114759</t>
+    <t>R58, R59, R64, R67</t>
+  </si>
+  <si>
+    <t>C138002</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 33Ohms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R58, R59, R64, R67</t>
-  </si>
-  <si>
-    <t>C138002</t>
+    <t>R68</t>
+  </si>
+  <si>
+    <t>C132157</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 12.1kOhms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R68</t>
-  </si>
-  <si>
-    <t>C132157</t>
+    <t>R71, R73, R74, R75, R76, R77</t>
+  </si>
+  <si>
+    <t>C105875</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 330Ohms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R71, R73, R74, R75, R76, R77</t>
-  </si>
-  <si>
-    <t>C105875</t>
+    <t>R78</t>
+  </si>
+  <si>
+    <t>C60491</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 100kOhms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R78</t>
-  </si>
-  <si>
-    <t>C60491</t>
+    <t>R80, R82, R84</t>
+  </si>
+  <si>
+    <t>C106231</t>
   </si>
   <si>
     <t>Thick Film Resistors - SMD General Purpose Chip Resistor 0402, 0Ohms, 1%, 1/16W</t>
   </si>
   <si>
-    <t>R80, R82, R84</t>
-  </si>
-  <si>
-    <t>C106231</t>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>C3012022</t>
   </si>
   <si>
     <t>Tactile Switches SMD OFF - (ON)</t>
   </si>
   <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>C3012022</t>
-  </si>
-  <si>
-    <t>Test point black, Mtg Hole 1.6, loop 3.2mm</t>
-  </si>
-  <si>
-    <t>TP4, TP5, TP6</t>
-  </si>
-  <si>
-    <t>C2906764</t>
+    <t>U3</t>
+  </si>
+  <si>
+    <t>C73631</t>
   </si>
   <si>
     <t>RS-485 Interface IC 5V-Supply</t>
   </si>
   <si>
-    <t>U3</t>
-  </si>
-  <si>
-    <t>C73631</t>
+    <t>U4, U10</t>
+  </si>
+  <si>
+    <t>C528656</t>
   </si>
   <si>
     <t>Digital Isolators 3.75 kV 5 forward &amp; 1 reverse 6-channel isolator</t>
   </si>
   <si>
-    <t>U4, U10</t>
-  </si>
-  <si>
-    <t>C528656</t>
+    <t>U5</t>
+  </si>
+  <si>
+    <t>C621424</t>
   </si>
   <si>
     <t>Ethernet PHY transceiver 10/100-Mbps</t>
   </si>
   <si>
-    <t>U5</t>
-  </si>
-  <si>
-    <t>C621424</t>
+    <t>U6</t>
+  </si>
+  <si>
+    <t>C36395</t>
   </si>
   <si>
     <t>LDO Voltage Regulators 3.3V 0.8A Positive</t>
   </si>
   <si>
-    <t>U6</t>
-  </si>
-  <si>
-    <t>C36395</t>
+    <t>U9</t>
+  </si>
+  <si>
+    <t>C20619634</t>
   </si>
   <si>
     <t>ARM Microcontrollers - MCU Arm Cortex-M33 32-bit 250 MHz 2 Mbytes Flash 640KB RAM I3C, DCMI, Ethernet, SMPS</t>
   </si>
   <si>
-    <t>U9</t>
-  </si>
-  <si>
-    <t>C20619634</t>
-  </si>
-  <si>
-    <t>Crystals 25MHz 6pF 25ppm -10C +70C</t>
-  </si>
-  <si>
     <t>Y1, Y3</t>
   </si>
   <si>
-    <t>C1669725</t>
+    <t>C91750</t>
+  </si>
+  <si>
+    <t>Crystals 25MHz 12pF 20ppm -40C +125C</t>
+  </si>
+  <si>
+    <t>Y2</t>
+  </si>
+  <si>
+    <t>C32346</t>
   </si>
   <si>
     <t>Crystals 32.768KHz 20ppm 12.5pF -40C +85C</t>
-  </si>
-  <si>
-    <t>Y2</t>
-  </si>
-  <si>
-    <t>C165064</t>
   </si>
 </sst>
 </file>
@@ -896,12 +878,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="12.75" baseColWidth="0"/>
   <cols>
-    <col min="1" max="1" width="70.09765625" customWidth="1"/>
-    <col min="2" max="2" width="25.41015625" customWidth="1"/>
-    <col min="3" max="3" width="26.7109375" customWidth="1"/>
+    <col min="1" max="1" width="20.2109375" customWidth="1"/>
+    <col min="2" max="2" width="18.421875" customWidth="1"/>
+    <col min="3" max="3" width="66.68359375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1617,28 +1599,6 @@
       </c>
       <c r="C65" s="16" t="s">
         <v>195</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3">
-      <c r="A66" s="25" t="s">
-        <v>196</v>
-      </c>
-      <c r="B66" s="16" t="s">
-        <v>197</v>
-      </c>
-      <c r="C66" s="16" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3">
-      <c r="A67" s="25" t="s">
-        <v>199</v>
-      </c>
-      <c r="B67" s="16" t="s">
-        <v>200</v>
-      </c>
-      <c r="C67" s="16" t="s">
-        <v>201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>